<commit_message>
saving old python version
</commit_message>
<xml_diff>
--- a/Briefing Data Pull Example.xlsx
+++ b/Briefing Data Pull Example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\seb0702\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wenxi/school/nu/PrepSummaries/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{C258E279-DAC5-4420-A727-16E90C51C421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="21660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contact Reports in the last 60 " sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
   <si>
     <t>Constituent: Donor ID</t>
   </si>
@@ -80,9 +80,6 @@
   </si>
   <si>
     <t>Email</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>N3038345</t>
@@ -159,11 +156,13 @@
       <sz val="12"/>
       <color rgb="FF56585B"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -602,14 +601,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="57" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
-    <col min="5" max="5" width="34.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="32" customWidth="1"/>
     <col min="8" max="8" width="38" customWidth="1"/>
     <col min="9" max="9" width="34" customWidth="1"/>
@@ -624,7 +623,7 @@
     <col min="18" max="18" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -638,10 +637,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>31</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>32</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
@@ -680,7 +679,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="217" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="221" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>1234567890</v>
       </c>
@@ -688,34 +687,34 @@
         <v>16</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L2" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="M2" s="5">
         <v>1365078.36</v>
@@ -727,51 +726,51 @@
         <v>46052</v>
       </c>
       <c r="P2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q2" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="R2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="Q2" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>22</v>
-      </c>
     </row>
-    <row r="3" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>1234567890</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>18</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>19</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="M3" s="5">
         <v>1365078.36</v>
@@ -783,13 +782,13 @@
         <v>46053</v>
       </c>
       <c r="P3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q3" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="R3" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="Q3" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>